<commit_message>
Feat/Style: Coloquei a coluna de série no excel, adicionei o app.route no app.py, e outras coisas
</commit_message>
<xml_diff>
--- a/Media_Alunos.escola.xlsx
+++ b/Media_Alunos.escola.xlsx
@@ -1,34 +1,97 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="204" yWindow="588" windowWidth="22716" windowHeight="8676"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Media </t>
+  </si>
+  <si>
+    <t>Frequencia</t>
+  </si>
+  <si>
+    <t>Ocorrencias</t>
+  </si>
+  <si>
+    <t>Baixa_renda</t>
+  </si>
+  <si>
+    <t>Trabalha</t>
+  </si>
+  <si>
+    <t>Nota1</t>
+  </si>
+  <si>
+    <t>Nota2</t>
+  </si>
+  <si>
+    <t>Nota3</t>
+  </si>
+  <si>
+    <t>Nota4</t>
+  </si>
+  <si>
+    <t>Nota5</t>
+  </si>
+  <si>
+    <t>Nota6</t>
+  </si>
+  <si>
+    <t>Joao</t>
+  </si>
+  <si>
+    <t>Maria</t>
+  </si>
+  <si>
+    <t>Carlos</t>
+  </si>
+  <si>
+    <t>Ana</t>
+  </si>
+  <si>
+    <t>Pedro</t>
+  </si>
+  <si>
+    <t>Jose</t>
+  </si>
+  <si>
+    <t>Teste</t>
+  </si>
+  <si>
+    <t>serie</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,80 +110,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,353 +404,338 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="2" width="9" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Nome</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Media </t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Frequencia</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Ocorrencias</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Baixa_renda</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Trabalha</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Nota1</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Nota2</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Nota3</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Nota4</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Nota5</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Nota6</t>
-        </is>
+    <row r="1" spans="1:13">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Joao</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="2" spans="1:13">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
         <v>8</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2">
         <v>75</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2">
         <v>2</v>
       </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2">
         <v>8</v>
       </c>
-      <c r="H2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I2" t="n">
+      <c r="I2">
+        <v>6</v>
+      </c>
+      <c r="J2">
         <v>4</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2">
         <v>2</v>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
         <v>3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Maria</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:13">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
         <v>5</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3">
         <v>70</v>
       </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="b">
+      <c r="E3">
         <v>0</v>
       </c>
       <c r="F3" t="b">
         <v>0</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3">
         <v>4</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3">
         <v>5</v>
       </c>
-      <c r="I3" t="n">
-        <v>6</v>
-      </c>
-      <c r="J3" t="n">
+      <c r="J3">
+        <v>6</v>
+      </c>
+      <c r="K3">
         <v>7</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3">
         <v>8</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3">
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Carlos</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:13">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
         <v>7</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4">
         <v>80</v>
       </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="b">
+      <c r="E4">
         <v>0</v>
       </c>
       <c r="F4" t="b">
         <v>0</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4">
         <v>7</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4">
         <v>5</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4">
         <v>4</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4">
         <v>3</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4">
         <v>2</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4">
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Ana</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>6</v>
-      </c>
-      <c r="C5" t="n">
+    <row r="5" spans="1:13">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5">
         <v>85</v>
       </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="b">
+      <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5">
         <v>5</v>
       </c>
-      <c r="H5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I5" t="n">
+      <c r="I5">
+        <v>6</v>
+      </c>
+      <c r="J5">
         <v>5</v>
       </c>
-      <c r="J5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K5" t="n">
+      <c r="K5">
+        <v>6</v>
+      </c>
+      <c r="L5">
         <v>7</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5">
         <v>8</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Pedro</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:13">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
         <v>4</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6">
         <v>60</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6">
         <v>3</v>
       </c>
-      <c r="E6" t="b">
-        <v>1</v>
-      </c>
       <c r="F6" t="b">
         <v>1</v>
       </c>
-      <c r="G6" t="n">
-        <v>6</v>
-      </c>
-      <c r="H6" t="n">
-        <v>6</v>
-      </c>
-      <c r="I6" t="n">
-        <v>6</v>
-      </c>
-      <c r="J6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K6" t="n">
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>6</v>
+      </c>
+      <c r="I6">
+        <v>6</v>
+      </c>
+      <c r="J6">
+        <v>6</v>
+      </c>
+      <c r="K6">
+        <v>6</v>
+      </c>
+      <c r="L6">
         <v>5</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6">
         <v>4</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Jose</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:13">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
         <v>5.8</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7">
         <v>80</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7">
         <v>3</v>
       </c>
-      <c r="E7" t="b">
-        <v>0</v>
-      </c>
       <c r="F7" t="b">
         <v>0</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7">
         <v>7</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7">
         <v>8</v>
       </c>
-      <c r="I7" t="n">
-        <v>6</v>
-      </c>
-      <c r="J7" t="n">
+      <c r="J7">
+        <v>6</v>
+      </c>
+      <c r="K7">
         <v>5</v>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
         <v>3</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Teste</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:13">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
         <v>7</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8">
         <v>90</v>
       </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="b">
+      <c r="E8">
         <v>1</v>
       </c>
       <c r="F8" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
         <v>4</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8">
         <v>4</v>
       </c>
-      <c r="J8" t="n">
-        <v>6</v>
-      </c>
-      <c r="K8" t="n">
+      <c r="K8">
+        <v>6</v>
+      </c>
+      <c r="L8">
         <v>10</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Co-authored-by: João Marcos <joaomarcosiewf@gmail.com>
</commit_message>
<xml_diff>
--- a/Media_Alunos.escola.xlsx
+++ b/Media_Alunos.escola.xlsx
@@ -457,7 +457,7 @@
         <v>12</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>8</v>
@@ -498,7 +498,7 @@
         <v>13</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C3">
         <v>5</v>
@@ -539,7 +539,7 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C4">
         <v>7</v>
@@ -580,7 +580,7 @@
         <v>15</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C5">
         <v>6</v>
@@ -621,7 +621,7 @@
         <v>16</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C6">
         <v>4</v>
@@ -662,7 +662,7 @@
         <v>17</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C7">
         <v>5.8</v>
@@ -703,7 +703,7 @@
         <v>18</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C8">
         <v>7</v>

</xml_diff>